<commit_message>
Added position for parties
</commit_message>
<xml_diff>
--- a/docs/ERD Documentation.xlsx
+++ b/docs/ERD Documentation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uoa-my.sharepoint.com/personal/ghin287_uoa_auckland_ac_nz/Documents/Documents/University/Datathon temp/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6BCFECDD-0F82-417B-BC2D-133351280788}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="8_{6BCFECDD-0F82-417B-BC2D-133351280788}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A5B61D4B-97F7-46C8-9C06-2473D564E6C9}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{61713979-96E7-4CAB-B837-6460B80500DB}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="100">
   <si>
     <t>Version</t>
   </si>
@@ -321,6 +321,24 @@
   </si>
   <si>
     <t>FK</t>
+  </si>
+  <si>
+    <t>position_id</t>
+  </si>
+  <si>
+    <t>Position</t>
+  </si>
+  <si>
+    <t>Whether a party is a defendant, accuser etc</t>
+  </si>
+  <si>
+    <t>position_name</t>
+  </si>
+  <si>
+    <t>What role this party is taking in the court</t>
+  </si>
+  <si>
+    <t>NOT IN ERD YET</t>
   </si>
 </sst>
 </file>
@@ -370,10 +388,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -708,7 +726,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{494E3E5D-6F4F-4225-ADF3-BF31FE81BED8}">
-  <dimension ref="A1:I91"/>
+  <dimension ref="A1:I98"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.21875" customWidth="1"/>
@@ -716,12 +734,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
       <c r="I1" s="1" t="s">
         <v>83</v>
       </c>
@@ -802,7 +820,7 @@
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A8" s="3" t="s">
+      <c r="A8" t="s">
         <v>8</v>
       </c>
       <c r="B8" t="s">
@@ -822,7 +840,7 @@
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A9" s="3" t="s">
+      <c r="A9" t="s">
         <v>14</v>
       </c>
       <c r="B9" t="s">
@@ -839,7 +857,7 @@
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" s="3" t="s">
+      <c r="A10" t="s">
         <v>17</v>
       </c>
       <c r="B10" t="s">
@@ -853,7 +871,7 @@
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A11" s="3" t="s">
+      <c r="A11" t="s">
         <v>19</v>
       </c>
       <c r="B11" t="s">
@@ -906,7 +924,7 @@
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A16" s="3" t="s">
+      <c r="A16" t="s">
         <v>17</v>
       </c>
       <c r="B16" t="s">
@@ -920,7 +938,7 @@
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="3" t="s">
+      <c r="A17" t="s">
         <v>25</v>
       </c>
       <c r="B17" t="s">
@@ -929,9 +947,6 @@
       <c r="E17" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="3"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
@@ -973,7 +988,7 @@
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A22" s="3" t="s">
+      <c r="A22" t="s">
         <v>19</v>
       </c>
       <c r="B22" t="s">
@@ -987,7 +1002,7 @@
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A23" s="3" t="s">
+      <c r="A23" t="s">
         <v>28</v>
       </c>
       <c r="B23" t="s">
@@ -1037,7 +1052,7 @@
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A28" s="3" t="s">
+      <c r="A28" t="s">
         <v>31</v>
       </c>
       <c r="B28" t="s">
@@ -1051,7 +1066,7 @@
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A29" s="3" t="s">
+      <c r="A29" t="s">
         <v>8</v>
       </c>
       <c r="B29" t="s">
@@ -1068,7 +1083,7 @@
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A30" s="3" t="s">
+      <c r="A30" t="s">
         <v>34</v>
       </c>
       <c r="B30" t="s">
@@ -1079,7 +1094,7 @@
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A31" s="3" t="s">
+      <c r="A31" t="s">
         <v>37</v>
       </c>
       <c r="B31" t="s">
@@ -1132,7 +1147,7 @@
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A36" s="3" t="s">
+      <c r="A36" t="s">
         <v>37</v>
       </c>
       <c r="B36" t="s">
@@ -1146,7 +1161,7 @@
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A37" s="3" t="s">
+      <c r="A37" t="s">
         <v>41</v>
       </c>
       <c r="B37" t="s">
@@ -1196,7 +1211,7 @@
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A42" s="3" t="s">
+      <c r="A42" t="s">
         <v>36</v>
       </c>
       <c r="B42" t="s">
@@ -1210,7 +1225,7 @@
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A43" s="3" t="s">
+      <c r="A43" t="s">
         <v>36</v>
       </c>
       <c r="B43" t="s">
@@ -1260,7 +1275,7 @@
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A48" s="3" t="s">
+      <c r="A48" t="s">
         <v>58</v>
       </c>
       <c r="B48" t="s">
@@ -1274,7 +1289,7 @@
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A49" s="3" t="s">
+      <c r="A49" t="s">
         <v>59</v>
       </c>
       <c r="B49" t="s">
@@ -1324,7 +1339,7 @@
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A55" s="3" t="s">
+      <c r="A55" t="s">
         <v>63</v>
       </c>
       <c r="B55" t="s">
@@ -1338,7 +1353,7 @@
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A56" s="3" t="s">
+      <c r="A56" t="s">
         <v>58</v>
       </c>
       <c r="B56" t="s">
@@ -1352,7 +1367,7 @@
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A57" s="3" t="s">
+      <c r="A57" t="s">
         <v>31</v>
       </c>
       <c r="B57" t="s">
@@ -1405,7 +1420,7 @@
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A62" s="3" t="s">
+      <c r="A62" t="s">
         <v>66</v>
       </c>
       <c r="B62" t="s">
@@ -1419,7 +1434,7 @@
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A63" s="3" t="s">
+      <c r="A63" t="s">
         <v>67</v>
       </c>
       <c r="B63" t="s">
@@ -1433,7 +1448,7 @@
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A64" s="3" t="s">
+      <c r="A64" t="s">
         <v>31</v>
       </c>
       <c r="B64" t="s">
@@ -1446,7 +1461,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66" s="1" t="s">
         <v>4</v>
       </c>
@@ -1457,7 +1472,7 @@
       <c r="D66" s="2"/>
       <c r="E66" s="2"/>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A67" s="1" t="s">
         <v>22</v>
       </c>
@@ -1468,7 +1483,7 @@
       <c r="D67" s="2"/>
       <c r="E67" s="2"/>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68" s="1" t="s">
         <v>5</v>
       </c>
@@ -1485,8 +1500,8 @@
         <v>42</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A69" s="3" t="s">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A69" t="s">
         <v>67</v>
       </c>
       <c r="B69" t="s">
@@ -1499,8 +1514,8 @@
         <v>13</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A70" s="3" t="s">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A70" t="s">
         <v>70</v>
       </c>
       <c r="B70" t="s">
@@ -1510,7 +1525,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A72" s="1" t="s">
         <v>4</v>
       </c>
@@ -1521,7 +1536,7 @@
       <c r="D72" s="2"/>
       <c r="E72" s="2"/>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A73" s="1" t="s">
         <v>22</v>
       </c>
@@ -1532,7 +1547,7 @@
       <c r="D73" s="2"/>
       <c r="E73" s="2"/>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A74" s="1" t="s">
         <v>5</v>
       </c>
@@ -1549,8 +1564,8 @@
         <v>42</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A75" s="3" t="s">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A75" t="s">
         <v>73</v>
       </c>
       <c r="B75" t="s">
@@ -1563,8 +1578,8 @@
         <v>13</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A76" s="3" t="s">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A76" t="s">
         <v>74</v>
       </c>
       <c r="B76" t="s">
@@ -1574,110 +1589,104 @@
         <v>76</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A78" s="1" t="s">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A77" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B77" t="s">
+        <v>9</v>
+      </c>
+      <c r="D77" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A78" s="4"/>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A79" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B78" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="C78" s="2"/>
-      <c r="D78" s="2"/>
-      <c r="E78" s="2"/>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A79" s="1" t="s">
-        <v>22</v>
-      </c>
       <c r="B79" s="2" t="s">
-        <v>78</v>
+        <v>95</v>
       </c>
       <c r="C79" s="2"/>
       <c r="D79" s="2"/>
       <c r="E79" s="2"/>
-    </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F79" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A80" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C80" s="2"/>
+      <c r="D80" s="2"/>
+      <c r="E80" s="2"/>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A81" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B80" s="1" t="s">
+      <c r="B81" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C80" s="1" t="s">
+      <c r="C81" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D80" s="1" t="s">
+      <c r="D81" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E80" s="1" t="s">
+      <c r="E81" s="1" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A81" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="B81" t="s">
-        <v>9</v>
-      </c>
-      <c r="C81" t="s">
-        <v>12</v>
-      </c>
-      <c r="D81" t="s">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A82" t="s">
+        <v>94</v>
+      </c>
+      <c r="B82" t="s">
+        <v>9</v>
+      </c>
+      <c r="C82" t="s">
+        <v>12</v>
+      </c>
+      <c r="D82" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A82" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="B82" t="s">
-        <v>9</v>
-      </c>
-      <c r="C82" t="s">
-        <v>12</v>
-      </c>
-      <c r="D82" t="s">
-        <v>93</v>
-      </c>
-    </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A83" s="3" t="s">
-        <v>73</v>
+      <c r="A83" t="s">
+        <v>97</v>
       </c>
       <c r="B83" t="s">
-        <v>9</v>
-      </c>
-      <c r="C83" t="s">
-        <v>12</v>
-      </c>
-      <c r="D83" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A84" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="B84" t="s">
-        <v>9</v>
-      </c>
-      <c r="C84" t="s">
-        <v>12</v>
-      </c>
-      <c r="D84" t="s">
-        <v>93</v>
-      </c>
-      <c r="E84" t="s">
-        <v>92</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="E83" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A85" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C85" s="2"/>
+      <c r="D85" s="2"/>
+      <c r="E85" s="2"/>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A86" s="1" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C86" s="2"/>
       <c r="D86" s="2"/>
@@ -1685,35 +1694,38 @@
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A87" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B87" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="C87" s="2"/>
-      <c r="D87" s="2"/>
-      <c r="E87" s="2"/>
+        <v>5</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C87" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D87" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E87" s="1" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A88" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B88" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C88" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D88" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E88" s="1" t="s">
-        <v>42</v>
+      <c r="A88" t="s">
+        <v>79</v>
+      </c>
+      <c r="B88" t="s">
+        <v>9</v>
+      </c>
+      <c r="C88" t="s">
+        <v>12</v>
+      </c>
+      <c r="D88" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A89" s="3" t="s">
-        <v>82</v>
+      <c r="A89" t="s">
+        <v>67</v>
       </c>
       <c r="B89" t="s">
         <v>9</v>
@@ -1722,11 +1734,11 @@
         <v>12</v>
       </c>
       <c r="D89" t="s">
-        <v>13</v>
+        <v>93</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A90" s="3" t="s">
+      <c r="A90" t="s">
         <v>73</v>
       </c>
       <c r="B90" t="s">
@@ -1740,8 +1752,8 @@
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A91" s="3" t="s">
-        <v>8</v>
+      <c r="A91" t="s">
+        <v>31</v>
       </c>
       <c r="B91" t="s">
         <v>9</v>
@@ -1752,24 +1764,96 @@
       <c r="D91" t="s">
         <v>93</v>
       </c>
+      <c r="E91" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A93" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B93" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C93" s="2"/>
+      <c r="D93" s="2"/>
+      <c r="E93" s="2"/>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A94" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B94" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C94" s="2"/>
+      <c r="D94" s="2"/>
+      <c r="E94" s="2"/>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A95" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B95" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C95" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D95" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E95" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A96" t="s">
+        <v>82</v>
+      </c>
+      <c r="B96" t="s">
+        <v>9</v>
+      </c>
+      <c r="C96" t="s">
+        <v>12</v>
+      </c>
+      <c r="D96" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A97" t="s">
+        <v>73</v>
+      </c>
+      <c r="B97" t="s">
+        <v>9</v>
+      </c>
+      <c r="C97" t="s">
+        <v>12</v>
+      </c>
+      <c r="D97" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A98" t="s">
+        <v>8</v>
+      </c>
+      <c r="B98" t="s">
+        <v>9</v>
+      </c>
+      <c r="C98" t="s">
+        <v>12</v>
+      </c>
+      <c r="D98" t="s">
+        <v>93</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="27">
-    <mergeCell ref="B78:E78"/>
+  <mergeCells count="29">
+    <mergeCell ref="A1:D1"/>
     <mergeCell ref="B79:E79"/>
-    <mergeCell ref="B86:E86"/>
-    <mergeCell ref="B87:E87"/>
-    <mergeCell ref="B59:E59"/>
-    <mergeCell ref="B60:E60"/>
-    <mergeCell ref="B66:E66"/>
-    <mergeCell ref="B67:E67"/>
-    <mergeCell ref="B72:E72"/>
-    <mergeCell ref="B73:E73"/>
-    <mergeCell ref="B39:E39"/>
-    <mergeCell ref="B40:E40"/>
-    <mergeCell ref="B45:E45"/>
-    <mergeCell ref="B46:E46"/>
-    <mergeCell ref="B52:E52"/>
+    <mergeCell ref="B80:E80"/>
     <mergeCell ref="B53:E53"/>
     <mergeCell ref="B34:E34"/>
     <mergeCell ref="B33:E33"/>
@@ -1781,7 +1865,21 @@
     <mergeCell ref="B20:E20"/>
     <mergeCell ref="B25:E25"/>
     <mergeCell ref="B26:E26"/>
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B39:E39"/>
+    <mergeCell ref="B40:E40"/>
+    <mergeCell ref="B45:E45"/>
+    <mergeCell ref="B46:E46"/>
+    <mergeCell ref="B52:E52"/>
+    <mergeCell ref="B85:E85"/>
+    <mergeCell ref="B86:E86"/>
+    <mergeCell ref="B93:E93"/>
+    <mergeCell ref="B94:E94"/>
+    <mergeCell ref="B59:E59"/>
+    <mergeCell ref="B60:E60"/>
+    <mergeCell ref="B66:E66"/>
+    <mergeCell ref="B67:E67"/>
+    <mergeCell ref="B72:E72"/>
+    <mergeCell ref="B73:E73"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>